<commit_message>
Include SLA value of Drymocallis arguta
</commit_message>
<xml_diff>
--- a/data/processed/data_processed_missing_20250902.xlsx
+++ b/data/processed/data_processed_missing_20250902.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -394,35 +394,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Drymocallis arguta</t>
+          <t>Symphyotrichum urophyllum</t>
         </is>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2">
-        <v>128</v>
-      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Rosaceae</t>
+          <t>Asteraceae</t>
         </is>
       </c>
       <c r="F2">
-        <v>0.91</v>
-      </c>
-      <c r="G2">
-        <v>0.000142</v>
+        <v>0.914</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Symphyotrichum urophyllum</t>
+          <t>Symphyotrichum pilosum</t>
         </is>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>157</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -430,20 +427,23 @@
         </is>
       </c>
       <c r="F3">
-        <v>0.914</v>
+        <v>0.91</v>
+      </c>
+      <c r="G3">
+        <v>0.000648</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Symphyotrichum pilosum</t>
+          <t>Euthamia graminifolia</t>
         </is>
       </c>
       <c r="B4">
         <v>0</v>
       </c>
       <c r="C4">
-        <v>157</v>
+        <v>134</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -451,196 +451,193 @@
         </is>
       </c>
       <c r="F4">
-        <v>0.91</v>
+        <v>0.6</v>
       </c>
       <c r="G4">
-        <v>0.000648</v>
+        <v>0.000106</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Euthamia graminifolia</t>
+          <t>Mollugo verticillata</t>
         </is>
       </c>
       <c r="B5">
         <v>0</v>
       </c>
       <c r="C5">
-        <v>134</v>
+        <v>97</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Asteraceae</t>
+          <t>Molluginaceae</t>
         </is>
       </c>
       <c r="F5">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="G5">
-        <v>0.000106</v>
+        <v>9.009999999999999E-05</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Mollugo verticillata</t>
+          <t>Phytolacca heterotepala</t>
         </is>
       </c>
       <c r="B6">
         <v>0</v>
       </c>
       <c r="C6">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Molluginaceae</t>
-        </is>
-      </c>
-      <c r="F6">
-        <v>0.2</v>
-      </c>
-      <c r="G6">
-        <v>9.009999999999999E-05</v>
+          <t>Phytolaccaceae</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Phytolacca heterotepala</t>
+          <t>Eragrostis spectabilis</t>
         </is>
       </c>
       <c r="B7">
         <v>0</v>
       </c>
       <c r="C7">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Phytolaccaceae</t>
-        </is>
+          <t>Poaceae</t>
+        </is>
+      </c>
+      <c r="F7">
+        <v>0.27</v>
+      </c>
+      <c r="G7">
+        <v>0.000257</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Eragrostis spectabilis</t>
+          <t>Phytolacca americana</t>
         </is>
       </c>
       <c r="B8">
         <v>0</v>
       </c>
       <c r="C8">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Poaceae</t>
+          <t>Phytolaccaceae</t>
         </is>
       </c>
       <c r="F8">
-        <v>0.27</v>
+        <v>2.425</v>
       </c>
       <c r="G8">
-        <v>0.000257</v>
+        <v>0.006869571</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Phytolacca americana</t>
+          <t>Panicum dichotomiflorum</t>
         </is>
       </c>
       <c r="B9">
         <v>0</v>
       </c>
       <c r="C9">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Phytolaccaceae</t>
+          <t>Poaceae</t>
         </is>
       </c>
       <c r="F9">
-        <v>2.425</v>
+        <v>0.7</v>
       </c>
       <c r="G9">
-        <v>0.006869571</v>
+        <v>0.000731</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Panicum dichotomiflorum</t>
+          <t>Taraxacum officinale</t>
         </is>
       </c>
       <c r="B10">
         <v>0</v>
       </c>
       <c r="C10">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Poaceae</t>
-        </is>
-      </c>
-      <c r="F10">
-        <v>0.7</v>
+          <t>Asteraceae</t>
+        </is>
       </c>
       <c r="G10">
-        <v>0.000731</v>
+        <v>0.0006827931029999999</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Taraxacum officinale</t>
+          <t>Verbena urticifolia</t>
         </is>
       </c>
       <c r="B11">
         <v>0</v>
       </c>
       <c r="C11">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Asteraceae</t>
+          <t>Verbenaceae</t>
         </is>
       </c>
       <c r="G11">
-        <v>0.0006827931029999999</v>
+        <v>0.00046</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Verbena urticifolia</t>
+          <t>Pseudognaphalium obtusifolium</t>
         </is>
       </c>
       <c r="B12">
         <v>0</v>
       </c>
       <c r="C12">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Verbenaceae</t>
+          <t>Asteraceae</t>
         </is>
       </c>
       <c r="G12">
-        <v>0.00046</v>
+        <v>3.8E-05</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Pseudognaphalium obtusifolium</t>
+          <t>Solidago altissima</t>
         </is>
       </c>
       <c r="B13">
@@ -655,220 +652,220 @@
         </is>
       </c>
       <c r="G13">
-        <v>3.8E-05</v>
+        <v>9.32E-05</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Solidago altissima</t>
+          <t>Paspalum setaceum</t>
         </is>
       </c>
       <c r="B14">
         <v>0</v>
       </c>
       <c r="C14">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Asteraceae</t>
+          <t>Poaceae</t>
         </is>
       </c>
       <c r="G14">
-        <v>9.32E-05</v>
+        <v>0.00098</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Paspalum setaceum</t>
+          <t>Toxicodendron radicans</t>
         </is>
       </c>
       <c r="B15">
         <v>0</v>
       </c>
       <c r="C15">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Poaceae</t>
+          <t>Anacardiaceae</t>
         </is>
       </c>
       <c r="G15">
-        <v>0.00098</v>
+        <v>0.01686</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Toxicodendron radicans</t>
+          <t>Bromus kalmii</t>
         </is>
       </c>
       <c r="B16">
         <v>0</v>
       </c>
       <c r="C16">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Anacardiaceae</t>
-        </is>
+          <t>Poaceae</t>
+        </is>
+      </c>
+      <c r="F16">
+        <v>0.91</v>
       </c>
       <c r="G16">
-        <v>0.01686</v>
+        <v>0.002497222</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Bromus kalmii</t>
+          <t>Morus alba</t>
         </is>
       </c>
       <c r="B17">
         <v>0</v>
       </c>
       <c r="C17">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Poaceae</t>
+          <t>Moraceae</t>
         </is>
       </c>
       <c r="F17">
-        <v>0.91</v>
+        <v>13</v>
       </c>
       <c r="G17">
-        <v>0.002497222</v>
+        <v>0.004701111</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Morus alba</t>
+          <t>Hypochaeris radicata</t>
         </is>
       </c>
       <c r="B18">
         <v>0</v>
       </c>
       <c r="C18">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Moraceae</t>
+          <t>Asteraceae</t>
         </is>
       </c>
       <c r="F18">
-        <v>13</v>
+        <v>0.32</v>
       </c>
       <c r="G18">
-        <v>0.004701111</v>
+        <v>0.0008140000000000001</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Hypochaeris radicata</t>
+          <t>Elaeagnus umbellata</t>
         </is>
       </c>
       <c r="B19">
         <v>0</v>
       </c>
       <c r="C19">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Asteraceae</t>
+          <t>Elaeagnaceae</t>
         </is>
       </c>
       <c r="F19">
-        <v>0.32</v>
+        <v>4.6</v>
       </c>
       <c r="G19">
-        <v>0.0008140000000000001</v>
+        <v>0.0152625</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Elaeagnus umbellata</t>
+          <t>Solanum americanum</t>
         </is>
       </c>
       <c r="B20">
         <v>0</v>
       </c>
       <c r="C20">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Elaeagnaceae</t>
+          <t>Solanaceae</t>
         </is>
       </c>
       <c r="F20">
-        <v>4.6</v>
+        <v>1</v>
       </c>
       <c r="G20">
-        <v>0.0152625</v>
+        <v>0.000859</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Solanum americanum</t>
+          <t>Fagopyrum esculentum</t>
         </is>
       </c>
       <c r="B21">
         <v>0</v>
       </c>
       <c r="C21">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Solanaceae</t>
+          <t>Polygonaceae</t>
         </is>
       </c>
       <c r="F21">
-        <v>1</v>
+        <v>0.828333333</v>
       </c>
       <c r="G21">
-        <v>0.000859</v>
+        <v>0.025273</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Fagopyrum esculentum</t>
+          <t>Danthonia spicata</t>
         </is>
       </c>
       <c r="B22">
         <v>0</v>
       </c>
       <c r="C22">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Polygonaceae</t>
-        </is>
-      </c>
-      <c r="F22">
-        <v>0.828333333</v>
+          <t>Poaceae</t>
+        </is>
       </c>
       <c r="G22">
-        <v>0.025273</v>
+        <v>0.000892</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Danthonia spicata</t>
+          <t>Morus rubra</t>
         </is>
       </c>
       <c r="B23">
@@ -879,41 +876,38 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Poaceae</t>
-        </is>
+          <t>Moraceae</t>
+        </is>
+      </c>
+      <c r="F23">
+        <v>20.56</v>
       </c>
       <c r="G23">
-        <v>0.000892</v>
+        <v>0.001448667</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Morus rubra</t>
+          <t>Cyperus lupulinus</t>
         </is>
       </c>
       <c r="B24">
         <v>0</v>
       </c>
       <c r="C24">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Moraceae</t>
-        </is>
-      </c>
-      <c r="F24">
-        <v>20.56</v>
-      </c>
-      <c r="G24">
-        <v>0.001448667</v>
+          <t>Cyperaceae</t>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Cyperus lupulinus</t>
+          <t>Elymus virginicus</t>
         </is>
       </c>
       <c r="B25">
@@ -924,62 +918,68 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Cyperaceae</t>
-        </is>
+          <t>Poaceae</t>
+        </is>
+      </c>
+      <c r="F25">
+        <v>0.76</v>
+      </c>
+      <c r="G25">
+        <v>0.004918556</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Elymus virginicus</t>
+          <t>Acer rubrum</t>
         </is>
       </c>
       <c r="B26">
         <v>0</v>
       </c>
       <c r="C26">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Poaceae</t>
+          <t>Sapindaceae</t>
         </is>
       </c>
       <c r="F26">
-        <v>0.76</v>
+        <v>24.52</v>
       </c>
       <c r="G26">
-        <v>0.004918556</v>
+        <v>0.019932063</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Acer rubrum</t>
+          <t>Geum canadense</t>
         </is>
       </c>
       <c r="B27">
         <v>0</v>
       </c>
       <c r="C27">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Sapindaceae</t>
+          <t>Rosaceae</t>
         </is>
       </c>
       <c r="F27">
-        <v>24.52</v>
+        <v>1.2</v>
       </c>
       <c r="G27">
-        <v>0.019932063</v>
+        <v>0.00515</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Geum canadense</t>
+          <t>Hackelia virginiana</t>
         </is>
       </c>
       <c r="B28">
@@ -990,20 +990,17 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Rosaceae</t>
-        </is>
-      </c>
-      <c r="F28">
-        <v>1.2</v>
+          <t>Boraginaceae</t>
+        </is>
       </c>
       <c r="G28">
-        <v>0.00515</v>
+        <v>0.0026</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Hackelia virginiana</t>
+          <t>Potentilla simplex</t>
         </is>
       </c>
       <c r="B29">
@@ -1014,17 +1011,14 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Boraginaceae</t>
-        </is>
-      </c>
-      <c r="G29">
-        <v>0.0026</v>
+          <t>Rosaceae</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Potentilla simplex</t>
+          <t>Pyrus calleryana</t>
         </is>
       </c>
       <c r="B30">
@@ -1038,11 +1032,17 @@
           <t>Rosaceae</t>
         </is>
       </c>
+      <c r="F30">
+        <v>6.5</v>
+      </c>
+      <c r="G30">
+        <v>0.0129</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Pyrus calleryana</t>
+          <t>Rubus occidentalis</t>
         </is>
       </c>
       <c r="B31">
@@ -1057,40 +1057,40 @@
         </is>
       </c>
       <c r="F31">
-        <v>6.5</v>
+        <v>1.8</v>
       </c>
       <c r="G31">
-        <v>0.0129</v>
+        <v>0.0013645</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Rubus occidentalis</t>
+          <t>Desmodium paniculatum</t>
         </is>
       </c>
       <c r="B32">
         <v>0</v>
       </c>
       <c r="C32">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Rosaceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="F32">
-        <v>1.8</v>
+        <v>0.91</v>
       </c>
       <c r="G32">
-        <v>0.0013645</v>
+        <v>0.00273</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Desmodium paniculatum</t>
+          <t>Euphorbia maculata</t>
         </is>
       </c>
       <c r="B33">
@@ -1101,20 +1101,17 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
-        </is>
-      </c>
-      <c r="F33">
-        <v>0.91</v>
+          <t>Euphorbiaceae</t>
+        </is>
       </c>
       <c r="G33">
-        <v>0.00273</v>
+        <v>0.000177</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Euphorbia maculata</t>
+          <t>Gamochaeta purpurea</t>
         </is>
       </c>
       <c r="B34">
@@ -1125,17 +1122,20 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Euphorbiaceae</t>
-        </is>
+          <t>Asteraceae</t>
+        </is>
+      </c>
+      <c r="F34">
+        <v>0.3</v>
       </c>
       <c r="G34">
-        <v>0.000177</v>
+        <v>3.83E-05</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Gamochaeta purpurea</t>
+          <t>Quercus velutina</t>
         </is>
       </c>
       <c r="B35">
@@ -1146,44 +1146,41 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Asteraceae</t>
+          <t>Fagaceae</t>
         </is>
       </c>
       <c r="F35">
-        <v>0.3</v>
+        <v>24.495</v>
       </c>
       <c r="G35">
-        <v>3.83E-05</v>
+        <v>1.851821111</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Quercus velutina</t>
+          <t>Asclepias amplexicaulis</t>
         </is>
       </c>
       <c r="B36">
         <v>0</v>
       </c>
       <c r="C36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Fagaceae</t>
-        </is>
-      </c>
-      <c r="F36">
-        <v>24.495</v>
+          <t>Apocynaceae</t>
+        </is>
       </c>
       <c r="G36">
-        <v>1.851821111</v>
+        <v>0.0106</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Asclepias amplexicaulis</t>
+          <t>Astragalus canadensis</t>
         </is>
       </c>
       <c r="B37">
@@ -1194,17 +1191,20 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Apocynaceae</t>
-        </is>
+          <t>Fabaceae</t>
+        </is>
+      </c>
+      <c r="F37">
+        <v>0.15</v>
       </c>
       <c r="G37">
-        <v>0.0106</v>
+        <v>0.001749667</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Astragalus canadensis</t>
+          <t>Circaea canadensis</t>
         </is>
       </c>
       <c r="B38">
@@ -1215,20 +1215,17 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
-        </is>
-      </c>
-      <c r="F38">
-        <v>0.15</v>
+          <t>Onagraceae</t>
+        </is>
       </c>
       <c r="G38">
-        <v>0.001749667</v>
+        <v>0.00264</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Circaea canadensis</t>
+          <t>Eragrostis cilianensis</t>
         </is>
       </c>
       <c r="B39">
@@ -1239,17 +1236,20 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Onagraceae</t>
-        </is>
+          <t>Poaceae</t>
+        </is>
+      </c>
+      <c r="F39">
+        <v>0.303333333</v>
       </c>
       <c r="G39">
-        <v>0.00264</v>
+        <v>7.13E-05</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Eragrostis cilianensis</t>
+          <t>Erechtites hieraciifolius</t>
         </is>
       </c>
       <c r="B40">
@@ -1260,20 +1260,17 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Poaceae</t>
-        </is>
-      </c>
-      <c r="F40">
-        <v>0.303333333</v>
+          <t>Asteraceae</t>
+        </is>
       </c>
       <c r="G40">
-        <v>7.13E-05</v>
+        <v>0.00056</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Erechtites hieraciifolius</t>
+          <t>Gleditsia triacanthos</t>
         </is>
       </c>
       <c r="B41">
@@ -1284,17 +1281,20 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Asteraceae</t>
-        </is>
+          <t>Fabaceae</t>
+        </is>
+      </c>
+      <c r="F41">
+        <v>27.16</v>
       </c>
       <c r="G41">
-        <v>0.00056</v>
+        <v>0.176454889</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Gleditsia triacanthos</t>
+          <t>Juncus dichotomus</t>
         </is>
       </c>
       <c r="B42">
@@ -1305,20 +1305,17 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Juncaceae</t>
         </is>
       </c>
       <c r="F42">
-        <v>27.16</v>
-      </c>
-      <c r="G42">
-        <v>0.176454889</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Juncus dichotomus</t>
+          <t>Lespedeza hirta</t>
         </is>
       </c>
       <c r="B43">
@@ -1329,17 +1326,20 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Juncaceae</t>
+          <t>Fabaceae</t>
         </is>
       </c>
       <c r="F43">
-        <v>0.88</v>
+        <v>1.8</v>
+      </c>
+      <c r="G43">
+        <v>0.0029105</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Lespedeza hirta</t>
+          <t>Lonicera maackii</t>
         </is>
       </c>
       <c r="B44">
@@ -1350,20 +1350,20 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Caprifoliaceae</t>
         </is>
       </c>
       <c r="F44">
-        <v>1.8</v>
+        <v>4.9</v>
       </c>
       <c r="G44">
-        <v>0.0029105</v>
+        <v>0.0030625</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Lonicera maackii</t>
+          <t>Scrophularia lanceolata</t>
         </is>
       </c>
       <c r="B45">
@@ -1374,20 +1374,20 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Caprifoliaceae</t>
+          <t>Scrophulariaceae</t>
         </is>
       </c>
       <c r="F45">
-        <v>4.9</v>
+        <v>1.5</v>
       </c>
       <c r="G45">
-        <v>0.0030625</v>
+        <v>0.000156</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Scrophularia lanceolata</t>
+          <t>Sporobolus heterolepis</t>
         </is>
       </c>
       <c r="B46">
@@ -1398,20 +1398,20 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Scrophulariaceae</t>
+          <t>Poaceae</t>
         </is>
       </c>
       <c r="F46">
-        <v>1.5</v>
+        <v>0.7</v>
       </c>
       <c r="G46">
-        <v>0.000156</v>
+        <v>0.0011365</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Sporobolus heterolepis</t>
+          <t>Symphyotrichum lanceolatum</t>
         </is>
       </c>
       <c r="B47">
@@ -1422,44 +1422,38 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Poaceae</t>
+          <t>Asteraceae</t>
         </is>
       </c>
       <c r="F47">
-        <v>0.7</v>
+        <v>1.8</v>
       </c>
       <c r="G47">
-        <v>0.0011365</v>
+        <v>0.000418</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Symphyotrichum lanceolatum</t>
+          <t>Digitaria cognata</t>
         </is>
       </c>
       <c r="B48">
         <v>0</v>
       </c>
-      <c r="C48">
-        <v>1</v>
-      </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Asteraceae</t>
-        </is>
-      </c>
-      <c r="F48">
-        <v>1.8</v>
+          <t>Poaceae</t>
+        </is>
       </c>
       <c r="G48">
-        <v>0.000418</v>
+        <v>0.00055</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Digitaria cognata</t>
+          <t>Melilotus albus</t>
         </is>
       </c>
       <c r="B49">
@@ -1467,17 +1461,20 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Poaceae</t>
-        </is>
+          <t>Fabaceae</t>
+        </is>
+      </c>
+      <c r="F49">
+        <v>1.5</v>
       </c>
       <c r="G49">
-        <v>0.00055</v>
+        <v>0.002233695</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Melilotus albus</t>
+          <t>Rhus typhina</t>
         </is>
       </c>
       <c r="B50">
@@ -1485,20 +1482,20 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Anacardiaceae</t>
         </is>
       </c>
       <c r="F50">
-        <v>1.5</v>
+        <v>7.28</v>
       </c>
       <c r="G50">
-        <v>0.002233695</v>
+        <v>0.0123925</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Rhus typhina</t>
+          <t>Ulmus pumila</t>
         </is>
       </c>
       <c r="B51">
@@ -1506,20 +1503,20 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Anacardiaceae</t>
+          <t>Ulmaceae</t>
         </is>
       </c>
       <c r="F51">
-        <v>7.28</v>
+        <v>21</v>
       </c>
       <c r="G51">
-        <v>0.0123925</v>
+        <v>0.006606584</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Ulmus pumila</t>
+          <t>Vitis aestivalis</t>
         </is>
       </c>
       <c r="B52">
@@ -1527,20 +1524,20 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Ulmaceae</t>
+          <t>Vitaceae</t>
         </is>
       </c>
       <c r="F52">
-        <v>21</v>
+        <v>9.1</v>
       </c>
       <c r="G52">
-        <v>0.006606584</v>
+        <v>0.0314525</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Vitis aestivalis</t>
+          <t>Vitis riparia</t>
         </is>
       </c>
       <c r="B53">
@@ -1552,30 +1549,9 @@
         </is>
       </c>
       <c r="F53">
-        <v>9.1</v>
+        <v>14</v>
       </c>
       <c r="G53">
-        <v>0.0314525</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Vitis riparia</t>
-        </is>
-      </c>
-      <c r="B54">
-        <v>0</v>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Vitaceae</t>
-        </is>
-      </c>
-      <c r="F54">
-        <v>14</v>
-      </c>
-      <c r="G54">
         <v>0.05514</v>
       </c>
     </row>

</xml_diff>